<commit_message>
completed testing of importing functions
also added vignette
</commit_message>
<xml_diff>
--- a/inst/extdata/example.xlsx
+++ b/inst/extdata/example.xlsx
@@ -10,7 +10,8 @@
     <sheet name="MB" sheetId="1" r:id="rId1"/>
     <sheet name="MP" sheetId="2" r:id="rId2"/>
     <sheet name="PH" sheetId="3" r:id="rId3"/>
-    <sheet name="FM" sheetId="4" r:id="rId4"/>
+    <sheet name="PB" sheetId="4" r:id="rId4"/>
+    <sheet name="FM" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2434,6 +2435,1315 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:BH7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>V6</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>V7</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>V8</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>V9</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>V10</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>V11</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>V12</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>V13</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>V14</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>V15</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>V16</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>V17</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>V18</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>V19</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>V20</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>V21</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>V22</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>V23</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>V24</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>V25</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>V26</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>V27</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>V28</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>V29</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>V30</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>V31</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>V32</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>V33</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>V34</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>V35</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>V36</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>V37</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>V38</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>V39</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>V40</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>V41</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>V42</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>V43</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>V44</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>V45</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>V46</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>V47</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>V48</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>V49</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>V50</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>V51</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>V52</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>V53</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>V54</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>V55</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>V56</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>V57</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>V58</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>V59</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>V60</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5050286</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>20120730</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5050286</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>20120806</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>5050297</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>20120103</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>5050297</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>20120226</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5050292</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>forensic psychiatry, exempt from BSCL since 01.07.2019</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>20121223</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>5050292</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>forensic psychiatry, exempt from BSCL since 01.07.2019</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>20121231</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>